<commit_message>
Log 10/11 long run, move strength to Thursdays, retarget plan to 4:45
- 10/11: 12.3 km long run with HR/pace/weather; 10/10 memo notes the Hyrox session
- Strength once a week on Thursdays (Hyrox or core), Monday notes cleared,
  10/12 becomes full rest with walking and foam rolling
- MP segments pinned to 6:40, long runs finish with a 6:45 block,
  peak long run 32 km with three checkpoints (11/8, 11/22, 12/9)
- Thursday rest days in Nov become 5 km recovery runs
- Site rebuilt from the workbook

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AidDHw4f5rLC2nZYJGxnSB
</commit_message>
<xml_diff>
--- a/富士山馬拉松_2026_課表.xlsx
+++ b/富士山馬拉松_2026_課表.xlsx
@@ -1094,7 +1094,7 @@
       </c>
       <c r="L4" s="51" t="inlineStr">
         <is>
-          <t>第一次成功壓住心拍的 Easy，GAP 7:03。第1km 6:23 偏快，後段心拍 141→156 微爬。路線爬升 91m 適合富士山</t>
+          <t>第一次成功壓住心拍的 Easy，GAP 7:03。第1km 6:23 偏快，後段心拍 141→156 微爬。路線爬升 91m 適合富士山 ／ 下午另做 Hyrox 58分（6站×2分），平均心拍152，難度9，隔天下半身痠痛</t>
         </is>
       </c>
       <c r="M4" s="50" t="inlineStr">
@@ -1173,18 +1173,54 @@
           <t>跑完記錄心拍，當基準</t>
         </is>
       </c>
-      <c r="J5" s="62" t="n"/>
-      <c r="K5" s="57" t="n"/>
-      <c r="L5" s="63" t="n"/>
-      <c r="M5" s="50" t="n"/>
-      <c r="N5" s="50" t="n"/>
-      <c r="O5" s="50" t="n"/>
-      <c r="P5" s="50" t="n"/>
-      <c r="Q5" s="50" t="n"/>
+      <c r="J5" s="62" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="K5" s="57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L5" s="63" t="inlineStr">
+        <is>
+          <t>第一次長跑。前半心拍146/後半152漂移+6，合格。前2km 7:19/7:13 偏快。4km處買水。前日Hyrox腿痠、27°C仍壓住心拍。基準線：27°C/HR149/7:40</t>
+        </is>
+      </c>
+      <c r="M5" s="50" t="inlineStr">
+        <is>
+          <t>1:36:09</t>
+        </is>
+      </c>
+      <c r="N5" s="50" t="inlineStr">
+        <is>
+          <t>7:47</t>
+        </is>
+      </c>
+      <c r="O5" s="50" t="n">
+        <v>149</v>
+      </c>
+      <c r="P5" s="50" t="n">
+        <v>162</v>
+      </c>
+      <c r="Q5" s="50" t="n">
+        <v>138</v>
+      </c>
       <c r="R5" s="50" t="n"/>
-      <c r="S5" s="50" t="n"/>
-      <c r="T5" s="50" t="n"/>
-      <c r="U5" s="50" t="n"/>
+      <c r="S5" s="50" t="inlineStr">
+        <is>
+          <t>晴 27°C / 體感 28°C / 濕度 46% / 北東風 10.4 km/h</t>
+        </is>
+      </c>
+      <c r="T5" s="50" t="inlineStr">
+        <is>
+          <t>Adidas EVO SL</t>
+        </is>
+      </c>
+      <c r="U5" s="50" t="inlineStr">
+        <is>
+          <t>Apple Watch Series 11</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="29.25" customHeight="1" s="43">
       <c r="A6" s="53" t="n">
@@ -1219,7 +1255,7 @@
       </c>
       <c r="I6" s="56" t="inlineStr">
         <is>
-          <t>休息日：15 分鐘核心＋臀腿（深蹲、臀橋、單腳硬舉、側平板）</t>
+          <t>完全休息。走路 20〜30 分 + 伸展滾筒（小腿／股四頭／臀）。腿痠散掉再跑</t>
         </is>
       </c>
       <c r="J6" s="50" t="n"/>
@@ -1370,7 +1406,7 @@
       </c>
       <c r="I9" s="56" t="inlineStr">
         <is>
-          <t>休息日：15 分鐘核心＋臀腿（深蹲、臀橋、單腳硬舉、側平板）</t>
+          <t>肌力日：Hyrox 或 15 分鐘核心＋臀腿 擇一，難度 6〜7，不要跑到心拍 160+</t>
         </is>
       </c>
       <c r="J9" s="50" t="n"/>
@@ -1560,11 +1596,7 @@
           <t>休息</t>
         </is>
       </c>
-      <c r="I13" s="56" t="inlineStr">
-        <is>
-          <t>休息日：15 分鐘核心＋臀腿（深蹲、臀橋、單腳硬舉、側平板）</t>
-        </is>
-      </c>
+      <c r="I13" s="56" t="n"/>
       <c r="J13" s="50" t="n"/>
       <c r="K13" s="53" t="n"/>
       <c r="L13" s="51" t="n"/>
@@ -1713,7 +1745,7 @@
       </c>
       <c r="I16" s="56" t="inlineStr">
         <is>
-          <t>休息日：15 分鐘核心＋臀腿（深蹲、臀橋、單腳硬舉、側平板）</t>
+          <t>肌力日：Hyrox 或 15 分鐘核心＋臀腿 擇一，難度 6〜7，不要跑到心拍 160+</t>
         </is>
       </c>
       <c r="J16" s="50" t="n"/>
@@ -1907,11 +1939,7 @@
           <t>休息</t>
         </is>
       </c>
-      <c r="I20" s="56" t="inlineStr">
-        <is>
-          <t>休息日：15 分鐘核心＋臀腿（深蹲、臀橋、單腳硬舉、側平板）</t>
-        </is>
-      </c>
+      <c r="I20" s="56" t="n"/>
       <c r="J20" s="50" t="n"/>
       <c r="K20" s="53" t="n"/>
       <c r="L20" s="51" t="n"/>
@@ -1997,7 +2025,7 @@
         </is>
       </c>
       <c r="F22" s="64" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G22" s="68" t="inlineStr">
         <is>
@@ -2006,7 +2034,7 @@
       </c>
       <c r="H22" s="68" t="inlineStr">
         <is>
-          <t>3 km Easy + 4 km @ MP + 1 km Easy</t>
+          <t>3 km Easy + 5 km @ 6:40 + 1 km Easy</t>
         </is>
       </c>
       <c r="I22" s="68" t="n"/>
@@ -2056,7 +2084,7 @@
       </c>
       <c r="I23" s="56" t="inlineStr">
         <is>
-          <t>休息日：15 分鐘核心＋臀腿（深蹲、臀橋、單腳硬舉、側平板）</t>
+          <t>肌力日：Hyrox 或 15 分鐘核心＋臀腿 擇一，難度 6〜7，不要跑到心拍 160+</t>
         </is>
       </c>
       <c r="J23" s="50" t="n"/>
@@ -2198,7 +2226,7 @@
       </c>
       <c r="H26" s="60" t="inlineStr">
         <is>
-          <t>長跑 18 km ★開始練補給</t>
+          <t>長跑 18 km，最後 4 km @ 6:45</t>
         </is>
       </c>
       <c r="I26" s="60" t="inlineStr">
@@ -2250,11 +2278,7 @@
           <t>休息</t>
         </is>
       </c>
-      <c r="I27" s="56" t="inlineStr">
-        <is>
-          <t>休息日：15 分鐘核心＋臀腿（深蹲、臀橋、單腳硬舉、側平板）</t>
-        </is>
-      </c>
+      <c r="I27" s="56" t="n"/>
       <c r="J27" s="50" t="n"/>
       <c r="K27" s="53" t="n"/>
       <c r="L27" s="51" t="n"/>
@@ -2385,21 +2409,25 @@
       </c>
       <c r="E30" s="55" t="inlineStr">
         <is>
-          <t>休息</t>
+          <t>Recovery</t>
         </is>
       </c>
       <c r="F30" s="53" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="56" t="n"/>
+        <v>5</v>
+      </c>
+      <c r="G30" s="56" t="inlineStr">
+        <is>
+          <t>心拍 ≤140</t>
+        </is>
+      </c>
       <c r="H30" s="56" t="inlineStr">
         <is>
-          <t>休息</t>
+          <t>恢復跑 4〜5 km（與肌力同日，兩者都輕）</t>
         </is>
       </c>
       <c r="I30" s="56" t="inlineStr">
         <is>
-          <t>休息日：15 分鐘核心＋臀腿（深蹲、臀橋、單腳硬舉、側平板）</t>
+          <t>肌力日：Hyrox 或 15 分鐘核心＋臀腿 擇一，難度 6〜7，不要跑到心拍 160+</t>
         </is>
       </c>
       <c r="J30" s="50" t="n"/>
@@ -2541,7 +2569,7 @@
       </c>
       <c r="H33" s="60" t="inlineStr">
         <is>
-          <t>長跑 22 km</t>
+          <t>長跑 22 km，最後 5 km @ 6:45 ★關卡1：最後5km穩6:45且心拍&lt;168才繼續下面的MP段</t>
         </is>
       </c>
       <c r="I33" s="60" t="inlineStr">
@@ -2593,11 +2621,7 @@
           <t>休息</t>
         </is>
       </c>
-      <c r="I34" s="56" t="inlineStr">
-        <is>
-          <t>休息日：15 分鐘核心＋臀腿（深蹲、臀橋、單腳硬舉、側平板）</t>
-        </is>
-      </c>
+      <c r="I34" s="56" t="n"/>
       <c r="J34" s="50" t="n"/>
       <c r="K34" s="53" t="n"/>
       <c r="L34" s="51" t="n"/>
@@ -2683,7 +2707,7 @@
         </is>
       </c>
       <c r="F36" s="64" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G36" s="68" t="inlineStr">
         <is>
@@ -2692,7 +2716,7 @@
       </c>
       <c r="H36" s="68" t="inlineStr">
         <is>
-          <t>2 km Easy + 6 km @ MP + 1 km Easy</t>
+          <t>2 km Easy + 7 km @ 6:40 + 1 km Easy</t>
         </is>
       </c>
       <c r="I36" s="67" t="inlineStr">
@@ -2732,21 +2756,25 @@
       </c>
       <c r="E37" s="55" t="inlineStr">
         <is>
-          <t>休息</t>
+          <t>Recovery</t>
         </is>
       </c>
       <c r="F37" s="53" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" s="56" t="n"/>
+        <v>5</v>
+      </c>
+      <c r="G37" s="56" t="inlineStr">
+        <is>
+          <t>心拍 ≤140</t>
+        </is>
+      </c>
       <c r="H37" s="56" t="inlineStr">
         <is>
-          <t>休息</t>
+          <t>恢復跑 4〜5 km（與肌力同日，兩者都輕）</t>
         </is>
       </c>
       <c r="I37" s="56" t="inlineStr">
         <is>
-          <t>休息日：15 分鐘核心＋臀腿（深蹲、臀橋、單腳硬舉、側平板）</t>
+          <t>肌力日：Hyrox 或 15 分鐘核心＋臀腿 擇一，難度 6〜7，不要跑到心拍 160+</t>
         </is>
       </c>
       <c r="J37" s="50" t="n"/>
@@ -2888,7 +2916,7 @@
       </c>
       <c r="H40" s="60" t="inlineStr">
         <is>
-          <t>長跑 26 km</t>
+          <t>長跑 26 km，最後 6 km @ 6:45</t>
         </is>
       </c>
       <c r="I40" s="60" t="inlineStr">
@@ -2940,11 +2968,7 @@
           <t>休息</t>
         </is>
       </c>
-      <c r="I41" s="56" t="inlineStr">
-        <is>
-          <t>休息日：15 分鐘核心＋臀腿（深蹲、臀橋、單腳硬舉、側平板）</t>
-        </is>
-      </c>
+      <c r="I41" s="56" t="n"/>
       <c r="J41" s="50" t="n"/>
       <c r="K41" s="53" t="n"/>
       <c r="L41" s="51" t="n"/>
@@ -3079,21 +3103,25 @@
       </c>
       <c r="E44" s="55" t="inlineStr">
         <is>
-          <t>休息</t>
+          <t>Recovery</t>
         </is>
       </c>
       <c r="F44" s="53" t="n">
-        <v>0</v>
-      </c>
-      <c r="G44" s="56" t="n"/>
+        <v>5</v>
+      </c>
+      <c r="G44" s="56" t="inlineStr">
+        <is>
+          <t>心拍 ≤140</t>
+        </is>
+      </c>
       <c r="H44" s="56" t="inlineStr">
         <is>
-          <t>休息</t>
+          <t>恢復跑 4〜5 km（與肌力同日，兩者都輕）</t>
         </is>
       </c>
       <c r="I44" s="56" t="inlineStr">
         <is>
-          <t>休息日：15 分鐘核心＋臀腿（深蹲、臀橋、單腳硬舉、側平板）</t>
+          <t>肌力日：Hyrox 或 15 分鐘核心＋臀腿 擇一，難度 6〜7，不要跑到心拍 160+</t>
         </is>
       </c>
       <c r="J44" s="50" t="n"/>
@@ -3226,7 +3254,7 @@
         </is>
       </c>
       <c r="F47" s="69" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G47" s="72" t="inlineStr">
         <is>
@@ -3235,12 +3263,12 @@
       </c>
       <c r="H47" s="72" t="inlineStr">
         <is>
-          <t>★ 峰值長跑 30 km（比賽預演）</t>
+          <t>★ 峰值長跑 32 km，最後 8 km @ 6:45（關卡1未過則維持 30 km 純 Easy）</t>
         </is>
       </c>
       <c r="I47" s="72" t="inlineStr">
         <is>
-          <t>比賽裝備、補給、起跑時間全部照比賽來。目標：完成且最後 5 km 心拍 &lt;170 還能控制 → 可試 5:00；否則比賽目標改 5:15〜5:30</t>
+          <t>★關卡2：最後8km穩6:45、心拍&lt;170、隔天無痛點 → 比賽配速6:40〜6:45；掉到7:15+ → 比賽7:00</t>
         </is>
       </c>
       <c r="J47" s="62" t="n"/>
@@ -3422,21 +3450,25 @@
       </c>
       <c r="E51" s="55" t="inlineStr">
         <is>
-          <t>休息</t>
+          <t>Recovery</t>
         </is>
       </c>
       <c r="F51" s="53" t="n">
-        <v>0</v>
-      </c>
-      <c r="G51" s="56" t="n"/>
+        <v>5</v>
+      </c>
+      <c r="G51" s="56" t="inlineStr">
+        <is>
+          <t>心拍 ≤140</t>
+        </is>
+      </c>
       <c r="H51" s="56" t="inlineStr">
         <is>
-          <t>休息</t>
+          <t>恢復跑 4〜5 km（與肌力同日，兩者都輕）</t>
         </is>
       </c>
       <c r="I51" s="56" t="inlineStr">
         <is>
-          <t>休息日：15 分鐘核心＋臀腿（深蹲、臀橋、單腳硬舉、側平板）</t>
+          <t>肌力日：Hyrox 或 15 分鐘核心＋臀腿 擇一，難度 6〜7，不要跑到心拍 160+</t>
         </is>
       </c>
       <c r="J51" s="50" t="n"/>
@@ -3630,11 +3662,7 @@
           <t>休息</t>
         </is>
       </c>
-      <c r="I55" s="56" t="inlineStr">
-        <is>
-          <t>休息日：15 分鐘核心＋臀腿（深蹲、臀橋、單腳硬舉、側平板）</t>
-        </is>
-      </c>
+      <c r="I55" s="56" t="n"/>
       <c r="J55" s="50" t="n"/>
       <c r="K55" s="53" t="n"/>
       <c r="L55" s="51" t="n"/>
@@ -3729,7 +3757,7 @@
       </c>
       <c r="H57" s="68" t="inlineStr">
         <is>
-          <t>3 km Easy + 3 km @ MP + 2 km Easy</t>
+          <t>3 km Easy + 4 km @ 6:40 + 2 km Easy</t>
         </is>
       </c>
       <c r="I57" s="67" t="inlineStr">
@@ -4071,7 +4099,11 @@
           <t>4 km Easy + 2 km @ MP</t>
         </is>
       </c>
-      <c r="I64" s="68" t="n"/>
+      <c r="I64" s="68" t="inlineStr">
+        <is>
+          <t>★關卡3：最後2km MP心拍&lt;165且體感輕 → 前半可押6:38；否則維持6:45</t>
+        </is>
+      </c>
       <c r="J64" s="50" t="n"/>
       <c r="K64" s="64" t="n"/>
       <c r="L64" s="51" t="n"/>

</xml_diff>

<commit_message>
Week 2: Hyrox on 10/17 replaces strength, 10/16 becomes recovery run
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AidDHw4f5rLC2nZYJGxnSB
</commit_message>
<xml_diff>
--- a/富士山馬拉松_2026_課表.xlsx
+++ b/富士山馬拉松_2026_課表.xlsx
@@ -1406,7 +1406,7 @@
       </c>
       <c r="I9" s="56" t="inlineStr">
         <is>
-          <t>肌力日：Hyrox 或 15 分鐘核心＋臀腿 擇一，難度 6〜7，不要跑到心拍 160+</t>
+          <t>休息。本週肌力由 10/17 Hyrox 取代，不做核心</t>
         </is>
       </c>
       <c r="J9" s="50" t="n"/>
@@ -1441,23 +1441,27 @@
       </c>
       <c r="E10" s="45" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Recovery</t>
         </is>
       </c>
       <c r="F10" s="45" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G10" s="49" t="inlineStr">
         <is>
-          <t>7:15〜7:45 / 心拍 140〜150</t>
+          <t>心拍 ≤140 / 7:45+</t>
         </is>
       </c>
       <c r="H10" s="48" t="inlineStr">
         <is>
-          <t>輕鬆跑 6 km</t>
-        </is>
-      </c>
-      <c r="I10" s="49" t="n"/>
+          <t>恢復跑 4 km</t>
+        </is>
+      </c>
+      <c r="I10" s="49" t="inlineStr">
+        <is>
+          <t>隔天 Hyrox，只活動腿，心拍超過 145 就走</t>
+        </is>
+      </c>
       <c r="J10" s="50" t="n"/>
       <c r="K10" s="45" t="n"/>
       <c r="L10" s="51" t="n"/>
@@ -1490,7 +1494,7 @@
       </c>
       <c r="E11" s="55" t="inlineStr">
         <is>
-          <t>休息</t>
+          <t>肌力</t>
         </is>
       </c>
       <c r="F11" s="53" t="n">
@@ -1499,10 +1503,14 @@
       <c r="G11" s="56" t="n"/>
       <c r="H11" s="56" t="inlineStr">
         <is>
-          <t>休息</t>
-        </is>
-      </c>
-      <c r="I11" s="56" t="n"/>
+          <t>Hyrox（已約）</t>
+        </is>
+      </c>
+      <c r="I11" s="56" t="inlineStr">
+        <is>
+          <t>難度 6〜7，站間休夠，心拍不衝 160+。這週肌力就是這場</t>
+        </is>
+      </c>
       <c r="J11" s="50" t="n"/>
       <c r="K11" s="53" t="n"/>
       <c r="L11" s="51" t="n"/>
@@ -1551,7 +1559,11 @@
           <t>長跑 14 km</t>
         </is>
       </c>
-      <c r="I12" s="61" t="n"/>
+      <c r="I12" s="61" t="inlineStr">
+        <is>
+          <t>前日 Hyrox。目標只有完成＋心拍 ≤150，配速掉到 8:00 也可。隔天腿痠 &gt;1 天＝Hyrox 強度太高</t>
+        </is>
+      </c>
       <c r="J12" s="62" t="n"/>
       <c r="K12" s="57" t="n"/>
       <c r="L12" s="63" t="n"/>

</xml_diff>

<commit_message>
Correct 10/11 long run to moving time and distance
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AidDHw4f5rLC2nZYJGxnSB
</commit_message>
<xml_diff>
--- a/富士山馬拉松_2026_課表.xlsx
+++ b/富士山馬拉松_2026_課表.xlsx
@@ -1174,7 +1174,7 @@
         </is>
       </c>
       <c r="J5" s="62" t="n">
-        <v>12.3</v>
+        <v>12</v>
       </c>
       <c r="K5" s="57" t="inlineStr">
         <is>
@@ -1183,17 +1183,17 @@
       </c>
       <c r="L5" s="63" t="inlineStr">
         <is>
-          <t>第一次長跑。前半心拍146/後半152漂移+6，合格。前2km 7:19/7:13 偏快。4km處買水。前日Hyrox腿痠、27°C仍壓住心拍。基準線：27°C/HR149/7:40</t>
+          <t>第一次長跑。前半心拍146/後半152漂移+6，合格。前2km 7:19/7:13 偏快。4km處買水。前日Hyrox腿痠、27°C仍壓住心拍。基準線：27°C/HR149/7:40；Strava 移動 1:36:09 含收操走路 0.3 km</t>
         </is>
       </c>
       <c r="M5" s="50" t="inlineStr">
         <is>
-          <t>1:36:09</t>
+          <t>1:31:07</t>
         </is>
       </c>
       <c r="N5" s="50" t="inlineStr">
         <is>
-          <t>7:47</t>
+          <t>7:36</t>
         </is>
       </c>
       <c r="O5" s="50" t="n">

</xml_diff>

<commit_message>
Verdicts are typed into the sheet; the page only renders them
Add columns V 判定 and W 提醒 to the workbook and fill the three logged
runs. build_site.py no longer judges distance, pace or heart rate; the
report card shows column V as the block title, coloured by its value, and
column W split on ｜ as the bullet list. README documents the update
command format.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AidDHw4f5rLC2nZYJGxnSB
</commit_message>
<xml_diff>
--- a/富士山馬拉松_2026_課表.xlsx
+++ b/富士山馬拉松_2026_課表.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="週總覽" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'課表'!$A$1:$U$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'課表'!$A$1:$W$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:U72"/>
+  <dimension ref="A1:W72"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="42" min="1" max="1"/>
@@ -803,6 +803,8 @@
     <col width="26" customWidth="1" style="42" min="19" max="19"/>
     <col width="14" customWidth="1" style="42" min="20" max="20"/>
     <col width="18" customWidth="1" style="42" min="21" max="21"/>
+    <col width="14" customWidth="1" style="43" min="22" max="22"/>
+    <col width="46" customWidth="1" style="43" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="43">
@@ -911,6 +913,16 @@
           <t>裝置</t>
         </is>
       </c>
+      <c r="V1" s="44" t="inlineStr">
+        <is>
+          <t>判定</t>
+        </is>
+      </c>
+      <c r="W1" s="44" t="inlineStr">
+        <is>
+          <t>提醒</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="43">
       <c r="A2" s="45" t="n">
@@ -1000,6 +1012,16 @@
       <c r="U2" s="50" t="inlineStr">
         <is>
           <t>Apple Watch Series 11</t>
+        </is>
+      </c>
+      <c r="V2" s="50" t="inlineStr">
+        <is>
+          <t>達成但有提醒</t>
+        </is>
+      </c>
+      <c r="W2" s="50" t="inlineStr">
+        <is>
+          <t>課表是 Easy，實際跑成 10K 配速｜心拍 169 超過上限 150 近 20</t>
         </is>
       </c>
     </row>
@@ -1047,6 +1069,8 @@
       <c r="S3" s="50" t="n"/>
       <c r="T3" s="50" t="n"/>
       <c r="U3" s="50" t="n"/>
+      <c r="V3" s="50" t="n"/>
+      <c r="W3" s="50" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1" s="43">
       <c r="A4" s="45" t="n">
@@ -1132,6 +1156,16 @@
           <t>Apple Watch Series 11</t>
         </is>
       </c>
+      <c r="V4" s="50" t="inlineStr">
+        <is>
+          <t>達成</t>
+        </is>
+      </c>
+      <c r="W4" s="50" t="inlineStr">
+        <is>
+          <t>第 1 km 6:23 起跑偏快，後段心拍 141→156 微爬</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="43">
       <c r="A5" s="57" t="n">
@@ -1219,6 +1253,16 @@
       <c r="U5" s="50" t="inlineStr">
         <is>
           <t>Apple Watch Series 11</t>
+        </is>
+      </c>
+      <c r="V5" s="50" t="inlineStr">
+        <is>
+          <t>達成</t>
+        </is>
+      </c>
+      <c r="W5" s="50" t="inlineStr">
+        <is>
+          <t>前 2 km 7:19/7:13 比要求的 7:45 快 30 秒｜最後 1 km 加速到 7:28、心拍 156，長跑最後不要加速</t>
         </is>
       </c>
     </row>
@@ -1270,6 +1314,8 @@
       <c r="S6" s="50" t="n"/>
       <c r="T6" s="50" t="n"/>
       <c r="U6" s="50" t="n"/>
+      <c r="V6" s="50" t="n"/>
+      <c r="W6" s="50" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="43">
       <c r="A7" s="45" t="n">
@@ -1319,6 +1365,8 @@
       <c r="S7" s="50" t="n"/>
       <c r="T7" s="50" t="n"/>
       <c r="U7" s="50" t="n"/>
+      <c r="V7" s="50" t="n"/>
+      <c r="W7" s="50" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="43">
       <c r="A8" s="64" t="n">
@@ -1372,6 +1420,8 @@
       <c r="S8" s="50" t="n"/>
       <c r="T8" s="50" t="n"/>
       <c r="U8" s="50" t="n"/>
+      <c r="V8" s="50" t="n"/>
+      <c r="W8" s="50" t="n"/>
     </row>
     <row r="9" ht="29.25" customHeight="1" s="43">
       <c r="A9" s="53" t="n">
@@ -1421,6 +1471,8 @@
       <c r="S9" s="50" t="n"/>
       <c r="T9" s="50" t="n"/>
       <c r="U9" s="50" t="n"/>
+      <c r="V9" s="50" t="n"/>
+      <c r="W9" s="50" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="43">
       <c r="A10" s="45" t="n">
@@ -1474,6 +1526,8 @@
       <c r="S10" s="50" t="n"/>
       <c r="T10" s="50" t="n"/>
       <c r="U10" s="50" t="n"/>
+      <c r="V10" s="50" t="n"/>
+      <c r="W10" s="50" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="43">
       <c r="A11" s="53" t="n">
@@ -1523,6 +1577,8 @@
       <c r="S11" s="50" t="n"/>
       <c r="T11" s="50" t="n"/>
       <c r="U11" s="50" t="n"/>
+      <c r="V11" s="50" t="n"/>
+      <c r="W11" s="50" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="43">
       <c r="A12" s="57" t="n">
@@ -1576,6 +1632,8 @@
       <c r="S12" s="50" t="n"/>
       <c r="T12" s="50" t="n"/>
       <c r="U12" s="50" t="n"/>
+      <c r="V12" s="50" t="n"/>
+      <c r="W12" s="50" t="n"/>
     </row>
     <row r="13" ht="29.25" customHeight="1" s="43">
       <c r="A13" s="53" t="n">
@@ -1621,6 +1679,8 @@
       <c r="S13" s="50" t="n"/>
       <c r="T13" s="50" t="n"/>
       <c r="U13" s="50" t="n"/>
+      <c r="V13" s="50" t="n"/>
+      <c r="W13" s="50" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="43">
       <c r="A14" s="45" t="n">
@@ -1670,6 +1730,8 @@
       <c r="S14" s="50" t="n"/>
       <c r="T14" s="50" t="n"/>
       <c r="U14" s="50" t="n"/>
+      <c r="V14" s="50" t="n"/>
+      <c r="W14" s="50" t="n"/>
     </row>
     <row r="15" ht="26.25" customHeight="1" s="43">
       <c r="A15" s="64" t="n">
@@ -1723,6 +1785,8 @@
       <c r="S15" s="50" t="n"/>
       <c r="T15" s="50" t="n"/>
       <c r="U15" s="50" t="n"/>
+      <c r="V15" s="50" t="n"/>
+      <c r="W15" s="50" t="n"/>
     </row>
     <row r="16" ht="29.25" customHeight="1" s="43">
       <c r="A16" s="53" t="n">
@@ -1772,6 +1836,8 @@
       <c r="S16" s="50" t="n"/>
       <c r="T16" s="50" t="n"/>
       <c r="U16" s="50" t="n"/>
+      <c r="V16" s="50" t="n"/>
+      <c r="W16" s="50" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="43">
       <c r="A17" s="45" t="n">
@@ -1821,6 +1887,8 @@
       <c r="S17" s="50" t="n"/>
       <c r="T17" s="50" t="n"/>
       <c r="U17" s="50" t="n"/>
+      <c r="V17" s="50" t="n"/>
+      <c r="W17" s="50" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="43">
       <c r="A18" s="53" t="n">
@@ -1866,6 +1934,8 @@
       <c r="S18" s="50" t="n"/>
       <c r="T18" s="50" t="n"/>
       <c r="U18" s="50" t="n"/>
+      <c r="V18" s="50" t="n"/>
+      <c r="W18" s="50" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="43">
       <c r="A19" s="57" t="n">
@@ -1919,6 +1989,8 @@
       <c r="S19" s="50" t="n"/>
       <c r="T19" s="50" t="n"/>
       <c r="U19" s="50" t="n"/>
+      <c r="V19" s="50" t="n"/>
+      <c r="W19" s="50" t="n"/>
     </row>
     <row r="20" ht="29.25" customHeight="1" s="43">
       <c r="A20" s="53" t="n">
@@ -1964,6 +2036,8 @@
       <c r="S20" s="50" t="n"/>
       <c r="T20" s="50" t="n"/>
       <c r="U20" s="50" t="n"/>
+      <c r="V20" s="50" t="n"/>
+      <c r="W20" s="50" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="43">
       <c r="A21" s="45" t="n">
@@ -2013,6 +2087,8 @@
       <c r="S21" s="50" t="n"/>
       <c r="T21" s="50" t="n"/>
       <c r="U21" s="50" t="n"/>
+      <c r="V21" s="50" t="n"/>
+      <c r="W21" s="50" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="43">
       <c r="A22" s="64" t="n">
@@ -2062,6 +2138,8 @@
       <c r="S22" s="50" t="n"/>
       <c r="T22" s="50" t="n"/>
       <c r="U22" s="50" t="n"/>
+      <c r="V22" s="50" t="n"/>
+      <c r="W22" s="50" t="n"/>
     </row>
     <row r="23" ht="29.25" customHeight="1" s="43">
       <c r="A23" s="53" t="n">
@@ -2111,6 +2189,8 @@
       <c r="S23" s="50" t="n"/>
       <c r="T23" s="50" t="n"/>
       <c r="U23" s="50" t="n"/>
+      <c r="V23" s="50" t="n"/>
+      <c r="W23" s="50" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="43">
       <c r="A24" s="45" t="n">
@@ -2160,6 +2240,8 @@
       <c r="S24" s="50" t="n"/>
       <c r="T24" s="50" t="n"/>
       <c r="U24" s="50" t="n"/>
+      <c r="V24" s="50" t="n"/>
+      <c r="W24" s="50" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="43">
       <c r="A25" s="53" t="n">
@@ -2205,6 +2287,8 @@
       <c r="S25" s="50" t="n"/>
       <c r="T25" s="50" t="n"/>
       <c r="U25" s="50" t="n"/>
+      <c r="V25" s="50" t="n"/>
+      <c r="W25" s="50" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="43">
       <c r="A26" s="57" t="n">
@@ -2258,6 +2342,8 @@
       <c r="S26" s="50" t="n"/>
       <c r="T26" s="50" t="n"/>
       <c r="U26" s="50" t="n"/>
+      <c r="V26" s="50" t="n"/>
+      <c r="W26" s="50" t="n"/>
     </row>
     <row r="27" ht="29.25" customHeight="1" s="43">
       <c r="A27" s="53" t="n">
@@ -2303,6 +2389,8 @@
       <c r="S27" s="50" t="n"/>
       <c r="T27" s="50" t="n"/>
       <c r="U27" s="50" t="n"/>
+      <c r="V27" s="50" t="n"/>
+      <c r="W27" s="50" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="43">
       <c r="A28" s="45" t="n">
@@ -2352,6 +2440,8 @@
       <c r="S28" s="50" t="n"/>
       <c r="T28" s="50" t="n"/>
       <c r="U28" s="50" t="n"/>
+      <c r="V28" s="50" t="n"/>
+      <c r="W28" s="50" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="43">
       <c r="A29" s="64" t="n">
@@ -2401,6 +2491,8 @@
       <c r="S29" s="50" t="n"/>
       <c r="T29" s="50" t="n"/>
       <c r="U29" s="50" t="n"/>
+      <c r="V29" s="50" t="n"/>
+      <c r="W29" s="50" t="n"/>
     </row>
     <row r="30" ht="29.25" customHeight="1" s="43">
       <c r="A30" s="53" t="n">
@@ -2454,6 +2546,8 @@
       <c r="S30" s="50" t="n"/>
       <c r="T30" s="50" t="n"/>
       <c r="U30" s="50" t="n"/>
+      <c r="V30" s="50" t="n"/>
+      <c r="W30" s="50" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1" s="43">
       <c r="A31" s="45" t="n">
@@ -2503,6 +2597,8 @@
       <c r="S31" s="50" t="n"/>
       <c r="T31" s="50" t="n"/>
       <c r="U31" s="50" t="n"/>
+      <c r="V31" s="50" t="n"/>
+      <c r="W31" s="50" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1" s="43">
       <c r="A32" s="53" t="n">
@@ -2548,6 +2644,8 @@
       <c r="S32" s="50" t="n"/>
       <c r="T32" s="50" t="n"/>
       <c r="U32" s="50" t="n"/>
+      <c r="V32" s="50" t="n"/>
+      <c r="W32" s="50" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1" s="43">
       <c r="A33" s="57" t="n">
@@ -2601,6 +2699,8 @@
       <c r="S33" s="50" t="n"/>
       <c r="T33" s="50" t="n"/>
       <c r="U33" s="50" t="n"/>
+      <c r="V33" s="50" t="n"/>
+      <c r="W33" s="50" t="n"/>
     </row>
     <row r="34" ht="29.25" customHeight="1" s="43">
       <c r="A34" s="53" t="n">
@@ -2646,6 +2746,8 @@
       <c r="S34" s="50" t="n"/>
       <c r="T34" s="50" t="n"/>
       <c r="U34" s="50" t="n"/>
+      <c r="V34" s="50" t="n"/>
+      <c r="W34" s="50" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="43">
       <c r="A35" s="45" t="n">
@@ -2695,6 +2797,8 @@
       <c r="S35" s="50" t="n"/>
       <c r="T35" s="50" t="n"/>
       <c r="U35" s="50" t="n"/>
+      <c r="V35" s="50" t="n"/>
+      <c r="W35" s="50" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="43">
       <c r="A36" s="64" t="n">
@@ -2748,6 +2852,8 @@
       <c r="S36" s="50" t="n"/>
       <c r="T36" s="50" t="n"/>
       <c r="U36" s="50" t="n"/>
+      <c r="V36" s="50" t="n"/>
+      <c r="W36" s="50" t="n"/>
     </row>
     <row r="37" ht="29.25" customHeight="1" s="43">
       <c r="A37" s="53" t="n">
@@ -2801,6 +2907,8 @@
       <c r="S37" s="50" t="n"/>
       <c r="T37" s="50" t="n"/>
       <c r="U37" s="50" t="n"/>
+      <c r="V37" s="50" t="n"/>
+      <c r="W37" s="50" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="43">
       <c r="A38" s="45" t="n">
@@ -2850,6 +2958,8 @@
       <c r="S38" s="50" t="n"/>
       <c r="T38" s="50" t="n"/>
       <c r="U38" s="50" t="n"/>
+      <c r="V38" s="50" t="n"/>
+      <c r="W38" s="50" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="43">
       <c r="A39" s="53" t="n">
@@ -2895,6 +3005,8 @@
       <c r="S39" s="50" t="n"/>
       <c r="T39" s="50" t="n"/>
       <c r="U39" s="50" t="n"/>
+      <c r="V39" s="50" t="n"/>
+      <c r="W39" s="50" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="43">
       <c r="A40" s="57" t="n">
@@ -2948,6 +3060,8 @@
       <c r="S40" s="50" t="n"/>
       <c r="T40" s="50" t="n"/>
       <c r="U40" s="50" t="n"/>
+      <c r="V40" s="50" t="n"/>
+      <c r="W40" s="50" t="n"/>
     </row>
     <row r="41" ht="29.25" customHeight="1" s="43">
       <c r="A41" s="53" t="n">
@@ -2993,6 +3107,8 @@
       <c r="S41" s="50" t="n"/>
       <c r="T41" s="50" t="n"/>
       <c r="U41" s="50" t="n"/>
+      <c r="V41" s="50" t="n"/>
+      <c r="W41" s="50" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="43">
       <c r="A42" s="45" t="n">
@@ -3042,6 +3158,8 @@
       <c r="S42" s="50" t="n"/>
       <c r="T42" s="50" t="n"/>
       <c r="U42" s="50" t="n"/>
+      <c r="V42" s="50" t="n"/>
+      <c r="W42" s="50" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1" s="43">
       <c r="A43" s="64" t="n">
@@ -3095,6 +3213,8 @@
       <c r="S43" s="50" t="n"/>
       <c r="T43" s="50" t="n"/>
       <c r="U43" s="50" t="n"/>
+      <c r="V43" s="50" t="n"/>
+      <c r="W43" s="50" t="n"/>
     </row>
     <row r="44" ht="29.25" customHeight="1" s="43">
       <c r="A44" s="53" t="n">
@@ -3148,6 +3268,8 @@
       <c r="S44" s="50" t="n"/>
       <c r="T44" s="50" t="n"/>
       <c r="U44" s="50" t="n"/>
+      <c r="V44" s="50" t="n"/>
+      <c r="W44" s="50" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1" s="43">
       <c r="A45" s="45" t="n">
@@ -3197,6 +3319,8 @@
       <c r="S45" s="50" t="n"/>
       <c r="T45" s="50" t="n"/>
       <c r="U45" s="50" t="n"/>
+      <c r="V45" s="50" t="n"/>
+      <c r="W45" s="50" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1" s="43">
       <c r="A46" s="53" t="n">
@@ -3242,6 +3366,8 @@
       <c r="S46" s="50" t="n"/>
       <c r="T46" s="50" t="n"/>
       <c r="U46" s="50" t="n"/>
+      <c r="V46" s="50" t="n"/>
+      <c r="W46" s="50" t="n"/>
     </row>
     <row r="47" ht="43.5" customHeight="1" s="43">
       <c r="A47" s="69" t="n">
@@ -3295,6 +3421,8 @@
       <c r="S47" s="50" t="n"/>
       <c r="T47" s="50" t="n"/>
       <c r="U47" s="50" t="n"/>
+      <c r="V47" s="50" t="n"/>
+      <c r="W47" s="50" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1" s="43">
       <c r="A48" s="53" t="n">
@@ -3344,6 +3472,8 @@
       <c r="S48" s="50" t="n"/>
       <c r="T48" s="50" t="n"/>
       <c r="U48" s="50" t="n"/>
+      <c r="V48" s="50" t="n"/>
+      <c r="W48" s="50" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1" s="43">
       <c r="A49" s="45" t="n">
@@ -3393,6 +3523,8 @@
       <c r="S49" s="50" t="n"/>
       <c r="T49" s="50" t="n"/>
       <c r="U49" s="50" t="n"/>
+      <c r="V49" s="50" t="n"/>
+      <c r="W49" s="50" t="n"/>
     </row>
     <row r="50" ht="15" customHeight="1" s="43">
       <c r="A50" s="45" t="n">
@@ -3442,6 +3574,8 @@
       <c r="S50" s="50" t="n"/>
       <c r="T50" s="50" t="n"/>
       <c r="U50" s="50" t="n"/>
+      <c r="V50" s="50" t="n"/>
+      <c r="W50" s="50" t="n"/>
     </row>
     <row r="51" ht="29.25" customHeight="1" s="43">
       <c r="A51" s="53" t="n">
@@ -3495,6 +3629,8 @@
       <c r="S51" s="50" t="n"/>
       <c r="T51" s="50" t="n"/>
       <c r="U51" s="50" t="n"/>
+      <c r="V51" s="50" t="n"/>
+      <c r="W51" s="50" t="n"/>
     </row>
     <row r="52" ht="15" customHeight="1" s="43">
       <c r="A52" s="45" t="n">
@@ -3544,6 +3680,8 @@
       <c r="S52" s="50" t="n"/>
       <c r="T52" s="50" t="n"/>
       <c r="U52" s="50" t="n"/>
+      <c r="V52" s="50" t="n"/>
+      <c r="W52" s="50" t="n"/>
     </row>
     <row r="53" ht="15" customHeight="1" s="43">
       <c r="A53" s="53" t="n">
@@ -3589,6 +3727,8 @@
       <c r="S53" s="50" t="n"/>
       <c r="T53" s="50" t="n"/>
       <c r="U53" s="50" t="n"/>
+      <c r="V53" s="50" t="n"/>
+      <c r="W53" s="50" t="n"/>
     </row>
     <row r="54" ht="26.25" customHeight="1" s="43">
       <c r="A54" s="57" t="n">
@@ -3642,6 +3782,8 @@
       <c r="S54" s="50" t="n"/>
       <c r="T54" s="50" t="n"/>
       <c r="U54" s="50" t="n"/>
+      <c r="V54" s="50" t="n"/>
+      <c r="W54" s="50" t="n"/>
     </row>
     <row r="55" ht="29.25" customHeight="1" s="43">
       <c r="A55" s="53" t="n">
@@ -3687,6 +3829,8 @@
       <c r="S55" s="50" t="n"/>
       <c r="T55" s="50" t="n"/>
       <c r="U55" s="50" t="n"/>
+      <c r="V55" s="50" t="n"/>
+      <c r="W55" s="50" t="n"/>
     </row>
     <row r="56" ht="15" customHeight="1" s="43">
       <c r="A56" s="45" t="n">
@@ -3736,6 +3880,8 @@
       <c r="S56" s="50" t="n"/>
       <c r="T56" s="50" t="n"/>
       <c r="U56" s="50" t="n"/>
+      <c r="V56" s="50" t="n"/>
+      <c r="W56" s="50" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1" s="43">
       <c r="A57" s="64" t="n">
@@ -3789,6 +3935,8 @@
       <c r="S57" s="50" t="n"/>
       <c r="T57" s="50" t="n"/>
       <c r="U57" s="50" t="n"/>
+      <c r="V57" s="50" t="n"/>
+      <c r="W57" s="50" t="n"/>
     </row>
     <row r="58" ht="15" customHeight="1" s="43">
       <c r="A58" s="53" t="n">
@@ -3834,6 +3982,8 @@
       <c r="S58" s="50" t="n"/>
       <c r="T58" s="50" t="n"/>
       <c r="U58" s="50" t="n"/>
+      <c r="V58" s="50" t="n"/>
+      <c r="W58" s="50" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1" s="43">
       <c r="A59" s="45" t="n">
@@ -3883,6 +4033,8 @@
       <c r="S59" s="50" t="n"/>
       <c r="T59" s="50" t="n"/>
       <c r="U59" s="50" t="n"/>
+      <c r="V59" s="50" t="n"/>
+      <c r="W59" s="50" t="n"/>
     </row>
     <row r="60" ht="15" customHeight="1" s="43">
       <c r="A60" s="53" t="n">
@@ -3928,6 +4080,8 @@
       <c r="S60" s="50" t="n"/>
       <c r="T60" s="50" t="n"/>
       <c r="U60" s="50" t="n"/>
+      <c r="V60" s="50" t="n"/>
+      <c r="W60" s="50" t="n"/>
     </row>
     <row r="61" ht="15" customHeight="1" s="43">
       <c r="A61" s="57" t="n">
@@ -3981,6 +4135,8 @@
       <c r="S61" s="50" t="n"/>
       <c r="T61" s="50" t="n"/>
       <c r="U61" s="50" t="n"/>
+      <c r="V61" s="50" t="n"/>
+      <c r="W61" s="50" t="n"/>
     </row>
     <row r="62" ht="15" customHeight="1" s="43">
       <c r="A62" s="53" t="n">
@@ -4026,6 +4182,8 @@
       <c r="S62" s="50" t="n"/>
       <c r="T62" s="50" t="n"/>
       <c r="U62" s="50" t="n"/>
+      <c r="V62" s="50" t="n"/>
+      <c r="W62" s="50" t="n"/>
     </row>
     <row r="63" ht="15" customHeight="1" s="43">
       <c r="A63" s="45" t="n">
@@ -4075,6 +4233,8 @@
       <c r="S63" s="50" t="n"/>
       <c r="T63" s="50" t="n"/>
       <c r="U63" s="50" t="n"/>
+      <c r="V63" s="50" t="n"/>
+      <c r="W63" s="50" t="n"/>
     </row>
     <row r="64" ht="15" customHeight="1" s="43">
       <c r="A64" s="64" t="n">
@@ -4128,6 +4288,8 @@
       <c r="S64" s="50" t="n"/>
       <c r="T64" s="50" t="n"/>
       <c r="U64" s="50" t="n"/>
+      <c r="V64" s="50" t="n"/>
+      <c r="W64" s="50" t="n"/>
     </row>
     <row r="65" ht="15" customHeight="1" s="43">
       <c r="A65" s="53" t="n">
@@ -4173,6 +4335,8 @@
       <c r="S65" s="50" t="n"/>
       <c r="T65" s="50" t="n"/>
       <c r="U65" s="50" t="n"/>
+      <c r="V65" s="50" t="n"/>
+      <c r="W65" s="50" t="n"/>
     </row>
     <row r="66" ht="15" customHeight="1" s="43">
       <c r="A66" s="64" t="n">
@@ -4226,6 +4390,8 @@
       <c r="S66" s="50" t="n"/>
       <c r="T66" s="50" t="n"/>
       <c r="U66" s="50" t="n"/>
+      <c r="V66" s="50" t="n"/>
+      <c r="W66" s="50" t="n"/>
     </row>
     <row r="67" ht="15" customHeight="1" s="43">
       <c r="A67" s="53" t="n">
@@ -4271,6 +4437,8 @@
       <c r="S67" s="50" t="n"/>
       <c r="T67" s="50" t="n"/>
       <c r="U67" s="50" t="n"/>
+      <c r="V67" s="50" t="n"/>
+      <c r="W67" s="50" t="n"/>
     </row>
     <row r="68" ht="15" customHeight="1" s="43">
       <c r="A68" s="53" t="n">
@@ -4320,6 +4488,8 @@
       <c r="S68" s="50" t="n"/>
       <c r="T68" s="50" t="n"/>
       <c r="U68" s="50" t="n"/>
+      <c r="V68" s="50" t="n"/>
+      <c r="W68" s="50" t="n"/>
     </row>
     <row r="69" ht="43.5" customHeight="1" s="43">
       <c r="A69" s="73" t="n">
@@ -4373,6 +4543,8 @@
       <c r="S69" s="50" t="n"/>
       <c r="T69" s="50" t="n"/>
       <c r="U69" s="50" t="n"/>
+      <c r="V69" s="50" t="n"/>
+      <c r="W69" s="50" t="n"/>
     </row>
     <row r="70"/>
     <row r="71" ht="15" customHeight="1" s="43">
@@ -4390,7 +4562,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U69"/>
+  <autoFilter ref="A1:W69"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Update week 7 and 8 focus text in the weekly overview
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AidDHw4f5rLC2nZYJGxnSB
</commit_message>
<xml_diff>
--- a/富士山馬拉松_2026_課表.xlsx
+++ b/富士山馬拉松_2026_課表.xlsx
@@ -4546,7 +4546,6 @@
       <c r="V69" s="50" t="n"/>
       <c r="W69" s="50" t="n"/>
     </row>
-    <row r="70"/>
     <row r="71" ht="15" customHeight="1" s="43">
       <c r="A71" s="77" t="inlineStr">
         <is>
@@ -4890,7 +4889,7 @@
       </c>
       <c r="I8" s="80" t="inlineStr">
         <is>
-          <t>★ 峰值 30 km 比賽預演</t>
+          <t>★ 峰值 32 km 比賽預演（關卡1未過則 30 km）</t>
         </is>
       </c>
     </row>
@@ -4927,7 +4926,7 @@
       </c>
       <c r="I9" s="80" t="inlineStr">
         <is>
-          <t>減量週，20 km 收尾 MP</t>
+          <t>減量週，20 km 最後 5 km MP</t>
         </is>
       </c>
     </row>
@@ -5042,6 +5041,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="15" customHeight="1" s="43">
       <c r="D14" s="83" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update 11/22 peak long run pace targets
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AidDHw4f5rLC2nZYJGxnSB
</commit_message>
<xml_diff>
--- a/富士山馬拉松_2026_課表.xlsx
+++ b/富士山馬拉松_2026_課表.xlsx
@@ -3396,7 +3396,7 @@
       </c>
       <c r="G47" s="72" t="inlineStr">
         <is>
-          <t>前 10 km 7:15〜7:30 / 中 7:00〜7:15 / 後 10 km 6:50〜7:10</t>
+          <t>前 12 km 7:15〜7:30 / 中 12 km 7:00〜7:15 / 最後 8 km 6:45</t>
         </is>
       </c>
       <c r="H47" s="72" t="inlineStr">
@@ -4546,6 +4546,7 @@
       <c r="V69" s="50" t="n"/>
       <c r="W69" s="50" t="n"/>
     </row>
+    <row r="70"/>
     <row r="71" ht="15" customHeight="1" s="43">
       <c r="A71" s="77" t="inlineStr">
         <is>
@@ -5041,7 +5042,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="15" customHeight="1" s="43">
       <c r="D14" s="83" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Log 10/13 Easy run (6.01 km)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AidDHw4f5rLC2nZYJGxnSB
</commit_message>
<xml_diff>
--- a/富士山馬拉松_2026_課表.xlsx
+++ b/富士山馬拉松_2026_課表.xlsx
@@ -1353,20 +1353,66 @@
         </is>
       </c>
       <c r="I7" s="49" t="n"/>
-      <c r="J7" s="50" t="n"/>
-      <c r="K7" s="45" t="n"/>
-      <c r="L7" s="51" t="n"/>
-      <c r="M7" s="50" t="n"/>
-      <c r="N7" s="50" t="n"/>
-      <c r="O7" s="50" t="n"/>
-      <c r="P7" s="50" t="n"/>
-      <c r="Q7" s="50" t="n"/>
-      <c r="R7" s="50" t="n"/>
-      <c r="S7" s="50" t="n"/>
-      <c r="T7" s="50" t="n"/>
-      <c r="U7" s="50" t="n"/>
-      <c r="V7" s="50" t="n"/>
-      <c r="W7" s="50" t="n"/>
+      <c r="J7" s="50" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="K7" s="45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L7" s="51" t="inlineStr">
+        <is>
+          <t>心拍控制最好的一次，第2km起幾乎水平。第1km 6:35 是心拍延遲（HR 132 時身體已在跑快）。第6km 8:01 是坡後自然放慢，正常。與10/10同配速心拍 150→140</t>
+        </is>
+      </c>
+      <c r="M7" s="50" t="inlineStr">
+        <is>
+          <t>44:36</t>
+        </is>
+      </c>
+      <c r="N7" s="50" t="inlineStr">
+        <is>
+          <t>7:25</t>
+        </is>
+      </c>
+      <c r="O7" s="50" t="n">
+        <v>140</v>
+      </c>
+      <c r="P7" s="50" t="n">
+        <v>148</v>
+      </c>
+      <c r="Q7" s="50" t="n">
+        <v>144</v>
+      </c>
+      <c r="R7" s="50" t="n">
+        <v>390</v>
+      </c>
+      <c r="S7" s="50" t="inlineStr">
+        <is>
+          <t>晴時多雲 23°C / 體感 24°C / 濕度 77% / 南東風 5.4 km/h</t>
+        </is>
+      </c>
+      <c r="T7" s="50" t="inlineStr">
+        <is>
+          <t>Adidas EVO SL</t>
+        </is>
+      </c>
+      <c r="U7" s="50" t="inlineStr">
+        <is>
+          <t>Apple Watch Series 11</t>
+        </is>
+      </c>
+      <c r="V7" s="50" t="inlineStr">
+        <is>
+          <t>達成</t>
+        </is>
+      </c>
+      <c r="W7" s="50" t="inlineStr">
+        <is>
+          <t>第 1 km 6:35 起跑偏快，心拍延遲造成；前 3 分鐘用呼吸不用錶</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="43">
       <c r="A8" s="64" t="n">

</xml_diff>

<commit_message>
Log 10/14 MP session (7.11 km)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AidDHw4f5rLC2nZYJGxnSB
</commit_message>
<xml_diff>
--- a/富士山馬拉松_2026_課表.xlsx
+++ b/富士山馬拉松_2026_課表.xlsx
@@ -1454,20 +1454,66 @@
           <t>MP 段心拍不要超過 165</t>
         </is>
       </c>
-      <c r="J8" s="50" t="n"/>
-      <c r="K8" s="64" t="n"/>
-      <c r="L8" s="51" t="n"/>
-      <c r="M8" s="50" t="n"/>
-      <c r="N8" s="50" t="n"/>
-      <c r="O8" s="50" t="n"/>
-      <c r="P8" s="50" t="n"/>
-      <c r="Q8" s="50" t="n"/>
-      <c r="R8" s="50" t="n"/>
-      <c r="S8" s="50" t="n"/>
-      <c r="T8" s="50" t="n"/>
-      <c r="U8" s="50" t="n"/>
-      <c r="V8" s="50" t="n"/>
-      <c r="W8" s="50" t="n"/>
+      <c r="J8" s="50" t="n">
+        <v>7.11</v>
+      </c>
+      <c r="K8" s="64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L8" s="51" t="inlineStr">
+        <is>
+          <t>第一次 MP 課。MP 段 6:16/6:23/6:29 心拍 152/157/157，比目標快 15〜20 秒但心拍餘裕大。收操心拍馬上回 148。6:40 比賽配速對心肺有餘裕，瓶頸在腿</t>
+        </is>
+      </c>
+      <c r="M8" s="50" t="inlineStr">
+        <is>
+          <t>50:28</t>
+        </is>
+      </c>
+      <c r="N8" s="50" t="inlineStr">
+        <is>
+          <t>7:06</t>
+        </is>
+      </c>
+      <c r="O8" s="50" t="n">
+        <v>146</v>
+      </c>
+      <c r="P8" s="50" t="n">
+        <v>161</v>
+      </c>
+      <c r="Q8" s="50" t="n">
+        <v>151</v>
+      </c>
+      <c r="R8" s="50" t="n">
+        <v>469</v>
+      </c>
+      <c r="S8" s="50" t="inlineStr">
+        <is>
+          <t>陰 23°C / 體感 23°C / 濕度 68% / 北北西風 5.8 km/h</t>
+        </is>
+      </c>
+      <c r="T8" s="50" t="inlineStr">
+        <is>
+          <t>Adidas EVO SL</t>
+        </is>
+      </c>
+      <c r="U8" s="50" t="inlineStr">
+        <is>
+          <t>Apple Watch Series 11</t>
+        </is>
+      </c>
+      <c r="V8" s="50" t="inlineStr">
+        <is>
+          <t>達成</t>
+        </is>
+      </c>
+      <c r="W8" s="50" t="inlineStr">
+        <is>
+          <t>MP 段跑成 6:20 而非 6:40，下次壓在 6:40〜6:45 練比賽配速感｜第 1 km 7:07 偏快</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="29.25" customHeight="1" s="43">
       <c r="A9" s="53" t="n">

</xml_diff>